<commit_message>
Receitas/Custos no modelo do BNB em PDF + correção do alinhamento do 'Ano Atual'
- receitas-bnb.pdf: formulário Receitas/Atividades reproduzido conforme o DESIGN_SPEC
  da skill (abas com Receitas/Custos ativa em laranja E87722, barra F08030, faixa da
  atividade, campos Descrição/Atividade Econômica, pares % de Utilização + Qtd. por
  ano com percentual em verde, zebra FFF8F0 e OBS em FFF2CC); A4 paisagem, 2 páginas
  (Ano Atual-Ano 5 e Ano 6-Ano 11, colunas fixas repetidas)
- CORREÇÃO: a coluna 'Ano Atual' recebia os dados do Ano 1 (deslocamento de uma
  coluna), mostrando produção para empresa que ainda não opera. Agora Ano Atual = 0%
  e a série Ano 1..Ano 11 fica alinhada; receitas-bnb.xlsx regenerado pelo gerador
  oficial com a mesma correção
- Valores conferidos: ano 1 R$ 2.750.000, ano 2 R$ 3.850.000, regime R$ 4.791.000

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CKyLR5v4criVdVXwyZSi7P
</commit_message>
<xml_diff>
--- a/estudo-mercado-gtk/dossie-bnb/receitas-bnb.xlsx
+++ b/estudo-mercado-gtk/dossie-bnb/receitas-bnb.xlsx
@@ -750,22 +750,22 @@
         <v>522655</v>
       </c>
       <c r="F11" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="13" t="n">
         <v>0.7175</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="I11" s="12" t="n">
         <v>375000</v>
       </c>
-      <c r="H11" s="13" t="n">
+      <c r="J11" s="13" t="n">
         <v>0.8929</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="K11" s="12" t="n">
         <v>466666.67</v>
-      </c>
-      <c r="J11" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="12" t="n">
-        <v>522654.55</v>
       </c>
       <c r="L11" s="13" t="n">
         <v>1</v>
@@ -843,22 +843,22 @@
         <v>276813</v>
       </c>
       <c r="F12" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="13" t="n">
         <v>0.4415</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="I12" s="12" t="n">
         <v>122222.22</v>
       </c>
-      <c r="H12" s="13" t="n">
+      <c r="J12" s="13" t="n">
         <v>0.7109000000000001</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="K12" s="12" t="n">
         <v>196777.78</v>
-      </c>
-      <c r="J12" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>276813.33</v>
       </c>
       <c r="L12" s="13" t="n">
         <v>1</v>
@@ -936,22 +936,22 @@
         <v>153996</v>
       </c>
       <c r="F13" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="13" t="n">
         <v>0.7015</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="I13" s="12" t="n">
         <v>108035.71</v>
       </c>
-      <c r="H13" s="13" t="n">
+      <c r="J13" s="13" t="n">
         <v>0.8929</v>
       </c>
-      <c r="I13" s="12" t="n">
+      <c r="K13" s="12" t="n">
         <v>137500</v>
-      </c>
-      <c r="J13" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K13" s="12" t="n">
-        <v>153996.43</v>
       </c>
       <c r="L13" s="13" t="n">
         <v>1</v>
@@ -1029,22 +1029,22 @@
         <v>34844</v>
       </c>
       <c r="F14" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="13" t="n">
         <v>0.4305</v>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="I14" s="12" t="n">
         <v>15000</v>
       </c>
-      <c r="H14" s="13" t="n">
+      <c r="J14" s="13" t="n">
         <v>0.7031000000000001</v>
       </c>
-      <c r="I14" s="12" t="n">
+      <c r="K14" s="12" t="n">
         <v>24500</v>
-      </c>
-      <c r="J14" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>34843.64</v>
       </c>
       <c r="L14" s="13" t="n">
         <v>1</v>
@@ -1122,22 +1122,22 @@
         <v>21013</v>
       </c>
       <c r="F15" s="13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="13" t="n">
         <v>0.4822</v>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="I15" s="12" t="n">
         <v>10131.58</v>
       </c>
-      <c r="H15" s="13" t="n">
+      <c r="J15" s="13" t="n">
         <v>0.7554000000000001</v>
       </c>
-      <c r="I15" s="12" t="n">
+      <c r="K15" s="12" t="n">
         <v>15872.81</v>
-      </c>
-      <c r="J15" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="12" t="n">
-        <v>21013.16</v>
       </c>
       <c r="L15" s="13" t="n">
         <v>1</v>
@@ -1197,7 +1197,7 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>OBS: Empresa em implantação: Qtd. Atual = 0 (sem operação). Qtd. Projetada = plano de regime (ano 3+), limitado ao teto de EPP (LC 123/2006) de R$ 4,8 milhões — receita de estabilização R$ 4.791.000. % de Utilização por ano reflete o ramp-up e a migração do mix para produtos de maior valor (vedação -&gt; estrutural e paver). Detalhamento mensal do ano 1 em previsao-faturamento.xlsx.</t>
+          <t>OBS: Empresa em implantação: coluna Ano Atual zerada (sem operação); Qtd. Atual = 0. Qtd. Projetada = plano de regime (Ano 3 em diante), limitado ao teto de EPP da LC 123/2006 — receita de estabilização de R$ 4.791.000. O % de Utilização por ano reflete o ramp-up comercial e a migração do mix para produtos de maior valor. Abertura mensal do Ano 1 em previsao-faturamento.pdf.</t>
         </is>
       </c>
     </row>

</xml_diff>